<commit_message>
Fix skill matching and match percentage bug
</commit_message>
<xml_diff>
--- a/backend/new.xlsx
+++ b/backend/new.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -410,6 +410,9 @@
         <v>Internship</v>
       </c>
       <c r="D1" t="str">
+        <v>enrollment</v>
+      </c>
+      <c r="E1" t="str">
         <v>Status</v>
       </c>
     </row>
@@ -424,12 +427,32 @@
         <v>new</v>
       </c>
       <c r="D2" t="str">
+        <v>No Enrollment</v>
+      </c>
+      <c r="E2" t="str">
         <v>Rejected</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>kii</v>
+      </c>
+      <c r="B3" t="str">
+        <v>kii@gmail.com</v>
+      </c>
+      <c r="C3" t="str">
+        <v>new</v>
+      </c>
+      <c r="D3" t="str">
+        <v>No Enrollment</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Approved</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>